<commit_message>
add tasks to scrub backlog
</commit_message>
<xml_diff>
--- a/scrum/TextTransformer.xlsx
+++ b/scrum/TextTransformer.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="54">
   <si>
     <t xml:space="preserve">Text Transformer</t>
   </si>
@@ -128,7 +128,7 @@
     <t xml:space="preserve">To be negotiated later</t>
   </si>
   <si>
-    <t xml:space="preserve">Sprint Goal:</t>
+    <t xml:space="preserve">Sprint Goal: Deliver working Text Transformer API with 9 Transformer Services</t>
   </si>
   <si>
     <t xml:space="preserve">Product Backlog Item</t>
@@ -189,6 +189,21 @@
   </si>
   <si>
     <t xml:space="preserve">Write the algorithm for removing repeated words</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Other]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setup logger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setup CI/CD to build docs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setup CI/CD to build JAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Draw UML</t>
   </si>
 </sst>
 </file>
@@ -851,7 +866,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:C36"/>
+  <dimension ref="A2:C41"/>
   <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="45.12"/>
@@ -859,7 +874,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="5" width="33"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
         <v>28</v>
       </c>
@@ -1034,6 +1049,31 @@
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="9" t="s">
         <v>40</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B39" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="4" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Sprint #1 backlog
</commit_message>
<xml_diff>
--- a/scrum/TextTransformer.xlsx
+++ b/scrum/TextTransformer.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="58">
   <si>
     <t xml:space="preserve">Text Transformer</t>
   </si>
@@ -137,13 +137,10 @@
     <t xml:space="preserve">Tasks</t>
   </si>
   <si>
-    <t xml:space="preserve">(for Product Backlog item)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Setup DTOs for data transfer from and to the controller</t>
   </si>
   <si>
-    <t xml:space="preserve">(for task)</t>
+    <t xml:space="preserve">15min</t>
   </si>
   <si>
     <t xml:space="preserve">Setup TransformationServiceRegistry</t>
@@ -170,12 +167,18 @@
     <t xml:space="preserve">Create ReverseTransformerService</t>
   </si>
   <si>
+    <t xml:space="preserve">30min</t>
+  </si>
+  <si>
     <t xml:space="preserve">Setup supported numbers swap list</t>
   </si>
   <si>
     <t xml:space="preserve">Create Nums2TextTransformerService</t>
   </si>
   <si>
+    <t xml:space="preserve">1.5h</t>
+  </si>
+  <si>
     <t xml:space="preserve">Setup supported acronyms </t>
   </si>
   <si>
@@ -188,9 +191,15 @@
     <t xml:space="preserve">Create LatexTransformerService</t>
   </si>
   <si>
+    <t xml:space="preserve">45min</t>
+  </si>
+  <si>
     <t xml:space="preserve">Write the algorithm for removing repeated words</t>
   </si>
   <si>
+    <t xml:space="preserve">2.5h</t>
+  </si>
+  <si>
     <t xml:space="preserve">[Other]</t>
   </si>
   <si>
@@ -204,6 +213,9 @@
   </si>
   <si>
     <t xml:space="preserve">Draw UML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20min</t>
   </si>
 </sst>
 </file>
@@ -703,7 +715,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="50.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
         <v>7</v>
       </c>
@@ -720,7 +732,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="86.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
         <v>10</v>
       </c>
@@ -737,7 +749,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="38.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
         <v>12</v>
       </c>
@@ -754,7 +766,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="38.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
         <v>14</v>
       </c>
@@ -771,7 +783,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="50.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
         <v>17</v>
       </c>
@@ -788,7 +800,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="62.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
         <v>19</v>
       </c>
@@ -822,7 +834,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="50.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
         <v>23</v>
       </c>
@@ -874,7 +886,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="5" width="33"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="26.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
         <v>28</v>
       </c>
@@ -890,190 +902,289 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="38.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
         <v>7</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="26.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="9" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="9" t="s">
+      <c r="C8" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="26.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="9" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C9" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="26.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
         <v>10</v>
       </c>
+      <c r="C11" s="5" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>39</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="26.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
         <v>12</v>
       </c>
+      <c r="C16" s="5" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>39</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="38.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
         <v>14</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="9" t="s">
         <v>42</v>
       </c>
+      <c r="C20" s="5" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="9" t="s">
         <v>43</v>
       </c>
+      <c r="C21" s="5" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>39</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="38.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
         <v>17</v>
       </c>
+      <c r="C23" s="5" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>39</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="38.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
         <v>19</v>
       </c>
+      <c r="C27" s="5" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>39</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="38.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
         <v>21</v>
       </c>
+      <c r="C31" s="5" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>39</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="38.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
         <v>23</v>
       </c>
+      <c r="C34" s="5" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="9" t="s">
-        <v>48</v>
+        <v>50</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="4" t="s">
-        <v>50</v>
+        <v>53</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="4" t="s">
-        <v>51</v>
+        <v>54</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="4" t="s">
-        <v>53</v>
+        <v>56</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add retro and new sprint backlog
</commit_message>
<xml_diff>
--- a/scrum/TextTransformer.xlsx
+++ b/scrum/TextTransformer.xlsx
@@ -5,12 +5,13 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Product Backlog" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Sprint #1 Backlog" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Sprint #2 Backlog" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="64">
   <si>
     <t xml:space="preserve">Text Transformer</t>
   </si>
@@ -216,6 +217,24 @@
   </si>
   <si>
     <t xml:space="preserve">20min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint Goal: Deliver working UI for Text Transformers and increase test coverage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create working UI for text transformers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create 20 unit tests methods for classes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create 15 mock objects in those unit tests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Write javadoc for 7 classes</t>
   </si>
 </sst>
 </file>
@@ -479,6 +498,17 @@
 </table>
 </file>
 
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela3_2" displayName="Tabela3_2" ref="A4:C44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A4:C44"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Product Backlog Item"/>
+    <tableColumn id="2" name="Tasks"/>
+    <tableColumn id="3" name="Labour intensity"/>
+  </tableColumns>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Motyw pakietu Office">
   <a:themeElements>
@@ -715,7 +745,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="50.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
         <v>7</v>
       </c>
@@ -732,7 +762,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="86.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
         <v>10</v>
       </c>
@@ -749,7 +779,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="38.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
         <v>12</v>
       </c>
@@ -766,7 +796,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="38.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
         <v>14</v>
       </c>
@@ -783,7 +813,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="50.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
         <v>17</v>
       </c>
@@ -800,7 +830,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="62.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
         <v>19</v>
       </c>
@@ -834,7 +864,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="50.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
         <v>23</v>
       </c>
@@ -886,7 +916,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="5" width="33"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="26.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
         <v>28</v>
       </c>
@@ -902,7 +932,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="38.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
         <v>7</v>
       </c>
@@ -926,7 +956,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="26.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="9" t="s">
         <v>34</v>
       </c>
@@ -934,7 +964,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="26.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="9" t="s">
         <v>35</v>
       </c>
@@ -942,7 +972,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="26.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
         <v>10</v>
       </c>
@@ -982,7 +1012,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="26.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
         <v>12</v>
       </c>
@@ -1006,7 +1036,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="38.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
         <v>14</v>
       </c>
@@ -1038,7 +1068,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="38.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
         <v>17</v>
       </c>
@@ -1070,7 +1100,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="38.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
         <v>19</v>
       </c>
@@ -1102,7 +1132,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="38.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
         <v>21</v>
       </c>
@@ -1126,7 +1156,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="38.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
         <v>23</v>
       </c>
@@ -1187,6 +1217,181 @@
         <v>57</v>
       </c>
     </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <tableParts>
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A2:C41"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="45.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="48.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="5" width="33"/>
+  </cols>
+  <sheetData>
+    <row r="2" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="9"/>
+    </row>
+    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9"/>
+      <c r="B11" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="9"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="9"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="9"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="9"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="9"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="9"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="9"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="9"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="9"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="9"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="9"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="9"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="9"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="9"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="9"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="9"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="9"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="9"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="9"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="9"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="9"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="9"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>